<commit_message>
Cosmetici: relações de entradas e saídas 09/2026 com a análise XML por XML (conferências, créditos, conta contábil)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GpFQAF7UfcTJUBPm398Z8s
</commit_message>
<xml_diff>
--- a/Cosmetici/Fiscal/2026-09/Relacao_Saidas_Cosmetici_09-2026.xlsx
+++ b/Cosmetici/Fiscal/2026-09/Relacao_Saidas_Cosmetici_09-2026.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Saídas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Saídas'!$A$4:$AA$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Saídas'!$A$4:$AC$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA109"/>
+  <dimension ref="A1:AC109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -517,7 +517,9 @@
     <col width="12" customWidth="1" min="24" max="24"/>
     <col width="22" customWidth="1" min="25" max="25"/>
     <col width="30" customWidth="1" min="26" max="26"/>
-    <col width="46" customWidth="1" min="27" max="27"/>
+    <col width="30" customWidth="1" min="27" max="27"/>
+    <col width="60" customWidth="1" min="28" max="28"/>
+    <col width="46" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -666,6 +668,16 @@
         </is>
       </c>
       <c r="AA4" s="3" t="inlineStr">
+        <is>
+          <t>Conferência XML x Faturamento x Registro (ERP)</t>
+        </is>
+      </c>
+      <c r="AB4" s="3" t="inlineStr">
+        <is>
+          <t>Análise (informativa - segue o XML)</t>
+        </is>
+      </c>
+      <c r="AC4" s="3" t="inlineStr">
         <is>
           <t>Chave de acesso</t>
         </is>
@@ -722,6 +734,12 @@
       </c>
       <c r="AA5" s="5" t="inlineStr">
         <is>
+          <t>número inutilizado - fora dos relatórios</t>
+        </is>
+      </c>
+      <c r="AB5" s="5" t="inlineStr"/>
+      <c r="AC5" s="5" t="inlineStr">
+        <is>
           <t>Protocolo 141260351772358</t>
         </is>
       </c>
@@ -825,6 +843,16 @@
       </c>
       <c r="AA6" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB6" s="5" t="inlineStr">
+        <is>
+          <t>[MÉDIA] Industrialização sem insumo: CFOP 5124 sem nota de remessa citada, sem retorno 5902/6902 e sem remessa recebida do cliente no mês - informativo (escriturado conforme o XML, CFOP 5124) | [MÉDIA] Diferimento 5124: 5124 para PR com CST 00 (ICMS R$ 108.44) enquanto 35 itens 5124 do mês saíram com diferimento (CST 51). Conferir se o diferimento se aplica a este cliente | [BAIXA] Grupo IPI: 2 it</t>
+        </is>
+      </c>
+      <c r="AC6" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089391000116135</t>
         </is>
       </c>
@@ -928,6 +956,12 @@
       </c>
       <c r="AA7" s="5" t="inlineStr">
         <is>
+          <t>cancelada - fora dos dois relatórios (filtro "Situação A")</t>
+        </is>
+      </c>
+      <c r="AB7" s="5" t="inlineStr"/>
+      <c r="AC7" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089401000115920</t>
         </is>
       </c>
@@ -1031,6 +1065,12 @@
       </c>
       <c r="AA8" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB8" s="5" t="inlineStr"/>
+      <c r="AC8" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089411000115935</t>
         </is>
       </c>
@@ -1134,6 +1174,12 @@
       </c>
       <c r="AA9" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB9" s="5" t="inlineStr"/>
+      <c r="AC9" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089421000115940</t>
         </is>
       </c>
@@ -1237,6 +1283,12 @@
       </c>
       <c r="AA10" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB10" s="5" t="inlineStr"/>
+      <c r="AC10" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089431000115891</t>
         </is>
       </c>
@@ -1340,6 +1392,12 @@
       </c>
       <c r="AA11" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB11" s="5" t="inlineStr"/>
+      <c r="AC11" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089441000115902</t>
         </is>
       </c>
@@ -1443,6 +1501,12 @@
       </c>
       <c r="AA12" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB12" s="5" t="inlineStr"/>
+      <c r="AC12" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089451000115918</t>
         </is>
       </c>
@@ -1546,6 +1610,12 @@
       </c>
       <c r="AA13" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB13" s="5" t="inlineStr"/>
+      <c r="AC13" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089461000196494</t>
         </is>
       </c>
@@ -1648,6 +1718,12 @@
         </is>
       </c>
       <c r="AA14" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB14" s="5" t="inlineStr"/>
+      <c r="AC14" s="5" t="inlineStr">
         <is>
           <t>41260933039048000162550010000089471000196505</t>
         </is>
@@ -1704,6 +1780,12 @@
       </c>
       <c r="AA15" s="5" t="inlineStr">
         <is>
+          <t>número inutilizado - fora dos relatórios</t>
+        </is>
+      </c>
+      <c r="AB15" s="5" t="inlineStr"/>
+      <c r="AC15" s="5" t="inlineStr">
+        <is>
           <t>Protocolo 141260353599070</t>
         </is>
       </c>
@@ -1807,6 +1889,12 @@
       </c>
       <c r="AA16" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB16" s="5" t="inlineStr"/>
+      <c r="AC16" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089491000204197</t>
         </is>
       </c>
@@ -1909,6 +1997,12 @@
         </is>
       </c>
       <c r="AA17" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB17" s="5" t="inlineStr"/>
+      <c r="AC17" s="5" t="inlineStr">
         <is>
           <t>41260933039048000162550010000089501000204201</t>
         </is>
@@ -1965,6 +2059,12 @@
       </c>
       <c r="AA18" s="5" t="inlineStr">
         <is>
+          <t>número inutilizado - fora dos relatórios</t>
+        </is>
+      </c>
+      <c r="AB18" s="5" t="inlineStr"/>
+      <c r="AC18" s="5" t="inlineStr">
+        <is>
           <t>Protocolo 141260353639120</t>
         </is>
       </c>
@@ -2068,6 +2168,12 @@
       </c>
       <c r="AA19" s="5" t="inlineStr">
         <is>
+          <t>cancelada - fora dos dois relatórios (filtro "Situação A")</t>
+        </is>
+      </c>
+      <c r="AB19" s="5" t="inlineStr"/>
+      <c r="AC19" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089521000162996</t>
         </is>
       </c>
@@ -2171,6 +2277,12 @@
       </c>
       <c r="AA20" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB20" s="5" t="inlineStr"/>
+      <c r="AC20" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089531000163000</t>
         </is>
       </c>
@@ -2274,6 +2386,12 @@
       </c>
       <c r="AA21" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB21" s="5" t="inlineStr"/>
+      <c r="AC21" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089541000163016</t>
         </is>
       </c>
@@ -2376,6 +2494,12 @@
         </is>
       </c>
       <c r="AA22" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB22" s="5" t="inlineStr"/>
+      <c r="AC22" s="5" t="inlineStr">
         <is>
           <t>41260933039048000162550010000089551000161819</t>
         </is>
@@ -2432,6 +2556,12 @@
       </c>
       <c r="AA23" s="5" t="inlineStr">
         <is>
+          <t>número inutilizado - fora dos relatórios</t>
+        </is>
+      </c>
+      <c r="AB23" s="5" t="inlineStr"/>
+      <c r="AC23" s="5" t="inlineStr">
+        <is>
           <t>Protocolo 141260355633030</t>
         </is>
       </c>
@@ -2535,6 +2665,12 @@
       </c>
       <c r="AA24" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB24" s="5" t="inlineStr"/>
+      <c r="AC24" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089571000162992</t>
         </is>
       </c>
@@ -2638,6 +2774,12 @@
       </c>
       <c r="AA25" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB25" s="5" t="inlineStr"/>
+      <c r="AC25" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089581000163007</t>
         </is>
       </c>
@@ -2741,6 +2883,12 @@
       </c>
       <c r="AA26" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB26" s="5" t="inlineStr"/>
+      <c r="AC26" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089591000156962</t>
         </is>
       </c>
@@ -2844,6 +2992,12 @@
       </c>
       <c r="AA27" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB27" s="5" t="inlineStr"/>
+      <c r="AC27" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089601000156971</t>
         </is>
       </c>
@@ -2947,6 +3101,12 @@
       </c>
       <c r="AA28" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB28" s="5" t="inlineStr"/>
+      <c r="AC28" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089611000197772</t>
         </is>
       </c>
@@ -3050,6 +3210,12 @@
       </c>
       <c r="AA29" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB29" s="5" t="inlineStr"/>
+      <c r="AC29" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089621000197788</t>
         </is>
       </c>
@@ -3153,6 +3319,12 @@
       </c>
       <c r="AA30" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB30" s="5" t="inlineStr"/>
+      <c r="AC30" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089631000118800</t>
         </is>
       </c>
@@ -3255,6 +3427,12 @@
         </is>
       </c>
       <c r="AA31" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB31" s="5" t="inlineStr"/>
+      <c r="AC31" s="5" t="inlineStr">
         <is>
           <t>41260933039048000162550010000089641000118815</t>
         </is>
@@ -3311,6 +3489,12 @@
       </c>
       <c r="AA32" s="5" t="inlineStr">
         <is>
+          <t>número inutilizado - fora dos relatórios</t>
+        </is>
+      </c>
+      <c r="AB32" s="5" t="inlineStr"/>
+      <c r="AC32" s="5" t="inlineStr">
+        <is>
           <t>Protocolo 141260363749669</t>
         </is>
       </c>
@@ -3414,6 +3598,12 @@
       </c>
       <c r="AA33" s="5" t="inlineStr">
         <is>
+          <t>Registro: UF PR x XML SP</t>
+        </is>
+      </c>
+      <c r="AB33" s="5" t="inlineStr"/>
+      <c r="AC33" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089661000161928</t>
         </is>
       </c>
@@ -3517,6 +3707,16 @@
       </c>
       <c r="AA34" s="5" t="inlineStr">
         <is>
+          <t>Registro: UF PR x XML SP</t>
+        </is>
+      </c>
+      <c r="AB34" s="5" t="inlineStr">
+        <is>
+          <t>[MÉDIA] CFOP revenda x produção: 1 item(ns) com CFOP 6102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+        </is>
+      </c>
+      <c r="AC34" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089671000161933</t>
         </is>
       </c>
@@ -3620,6 +3820,12 @@
       </c>
       <c r="AA35" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB35" s="5" t="inlineStr"/>
+      <c r="AC35" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089681000161949</t>
         </is>
       </c>
@@ -3723,6 +3929,16 @@
       </c>
       <c r="AA36" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB36" s="5" t="inlineStr">
+        <is>
+          <t>[MÉDIA] CFOP revenda x produção: 2 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+        </is>
+      </c>
+      <c r="AC36" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089691000161954</t>
         </is>
       </c>
@@ -3826,6 +4042,12 @@
       </c>
       <c r="AA37" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB37" s="5" t="inlineStr"/>
+      <c r="AC37" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089701000116445</t>
         </is>
       </c>
@@ -3929,6 +4151,12 @@
       </c>
       <c r="AA38" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB38" s="5" t="inlineStr"/>
+      <c r="AC38" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089711000207812</t>
         </is>
       </c>
@@ -4032,6 +4260,16 @@
       </c>
       <c r="AA39" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB39" s="5" t="inlineStr">
+        <is>
+          <t>[BAIXA] Grupo IPI: 2 item(ns) de produto (CFOP 6124) sem grupo de IPI (CST) - conferir o cadastro do produto no ERP</t>
+        </is>
+      </c>
+      <c r="AC39" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089731000116625</t>
         </is>
       </c>
@@ -4135,6 +4373,12 @@
       </c>
       <c r="AA40" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB40" s="5" t="inlineStr"/>
+      <c r="AC40" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089741000116630</t>
         </is>
       </c>
@@ -4238,6 +4482,12 @@
       </c>
       <c r="AA41" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB41" s="5" t="inlineStr"/>
+      <c r="AC41" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089751000191575</t>
         </is>
       </c>
@@ -4341,6 +4591,12 @@
       </c>
       <c r="AA42" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB42" s="5" t="inlineStr"/>
+      <c r="AC42" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089761000191580</t>
         </is>
       </c>
@@ -4444,6 +4700,12 @@
       </c>
       <c r="AA43" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB43" s="5" t="inlineStr"/>
+      <c r="AC43" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089771000191596</t>
         </is>
       </c>
@@ -4546,6 +4808,16 @@
         </is>
       </c>
       <c r="AA44" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB44" s="5" t="inlineStr">
+        <is>
+          <t>[MÉDIA] CFOP revenda x produção: 9 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+        </is>
+      </c>
+      <c r="AC44" s="5" t="inlineStr">
         <is>
           <t>41260933039048000162550010000089781000162046</t>
         </is>
@@ -4602,6 +4874,12 @@
       </c>
       <c r="AA45" s="5" t="inlineStr">
         <is>
+          <t>número inutilizado - fora dos relatórios</t>
+        </is>
+      </c>
+      <c r="AB45" s="5" t="inlineStr"/>
+      <c r="AC45" s="5" t="inlineStr">
+        <is>
           <t>Protocolo 141260375536433</t>
         </is>
       </c>
@@ -4705,6 +4983,16 @@
       </c>
       <c r="AA46" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB46" s="5" t="inlineStr">
+        <is>
+          <t>[MÉDIA] Industrialização sem insumo: CFOP 6124 sem nota de remessa citada, sem retorno 5902/6902 e sem remessa recebida do cliente no mês - informativo (escriturado conforme o XML, CFOP 6124)</t>
+        </is>
+      </c>
+      <c r="AC46" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089791000217000</t>
         </is>
       </c>
@@ -4808,6 +5096,16 @@
       </c>
       <c r="AA47" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB47" s="5" t="inlineStr">
+        <is>
+          <t>[MÉDIA] CFOP revenda x produção: 19 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS" | [BAIXA] Grupo IPI: 3 item(ns) de produto (CFOP 5102) sem grupo de IPI (CST) - conferir o cadastro do produto no ERP</t>
+        </is>
+      </c>
+      <c r="AC47" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089801000162060</t>
         </is>
       </c>
@@ -4911,6 +5209,16 @@
       </c>
       <c r="AA48" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB48" s="5" t="inlineStr">
+        <is>
+          <t>[MÉDIA] CFOP revenda x produção: 1 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+        </is>
+      </c>
+      <c r="AC48" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089811000162076</t>
         </is>
       </c>
@@ -5014,6 +5322,16 @@
       </c>
       <c r="AA49" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB49" s="5" t="inlineStr">
+        <is>
+          <t>[MÉDIA] CFOP revenda x produção: 1 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+        </is>
+      </c>
+      <c r="AC49" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089821000162081</t>
         </is>
       </c>
@@ -5117,6 +5435,12 @@
       </c>
       <c r="AA50" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB50" s="5" t="inlineStr"/>
+      <c r="AC50" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089831000120041</t>
         </is>
       </c>
@@ -5220,6 +5544,12 @@
       </c>
       <c r="AA51" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB51" s="5" t="inlineStr"/>
+      <c r="AC51" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089841000120057</t>
         </is>
       </c>
@@ -5323,6 +5653,12 @@
       </c>
       <c r="AA52" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB52" s="5" t="inlineStr"/>
+      <c r="AC52" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089851000116375</t>
         </is>
       </c>
@@ -5426,6 +5762,12 @@
       </c>
       <c r="AA53" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB53" s="5" t="inlineStr"/>
+      <c r="AC53" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089861000116380</t>
         </is>
       </c>
@@ -5529,6 +5871,12 @@
       </c>
       <c r="AA54" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB54" s="5" t="inlineStr"/>
+      <c r="AC54" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089871000126294</t>
         </is>
       </c>
@@ -5632,6 +5980,12 @@
       </c>
       <c r="AA55" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB55" s="5" t="inlineStr"/>
+      <c r="AC55" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089881000126305</t>
         </is>
       </c>
@@ -5735,6 +6089,16 @@
       </c>
       <c r="AA56" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB56" s="5" t="inlineStr">
+        <is>
+          <t>[ALTA] Industrialização x retorno: Item 1 (FRASCO IMPRESSO OX 30V 900ML MIX ETERNIZE) é insumo do cliente (CST 41, PIS 49) com CFOP 5124 de industrialização - o mesmo item foi devolvido também na NF 8993 (5902). Retorno de insumo é 5902/6902; como está, R$ 600.00 entra no acumulador de industrialização e na base do PIS/COFINS e do IRPJ/CSLL</t>
+        </is>
+      </c>
+      <c r="AC56" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089891000116358</t>
         </is>
       </c>
@@ -5838,6 +6202,12 @@
       </c>
       <c r="AA57" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB57" s="5" t="inlineStr"/>
+      <c r="AC57" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089901000207184</t>
         </is>
       </c>
@@ -5941,6 +6311,12 @@
       </c>
       <c r="AA58" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB58" s="5" t="inlineStr"/>
+      <c r="AC58" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089911000207190</t>
         </is>
       </c>
@@ -6044,6 +6420,12 @@
       </c>
       <c r="AA59" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB59" s="5" t="inlineStr"/>
+      <c r="AC59" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089921000116388</t>
         </is>
       </c>
@@ -6147,6 +6529,12 @@
       </c>
       <c r="AA60" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB60" s="5" t="inlineStr"/>
+      <c r="AC60" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089931000116393</t>
         </is>
       </c>
@@ -6250,6 +6638,12 @@
       </c>
       <c r="AA61" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB61" s="5" t="inlineStr"/>
+      <c r="AC61" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089941000166452</t>
         </is>
       </c>
@@ -6353,6 +6747,12 @@
       </c>
       <c r="AA62" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB62" s="5" t="inlineStr"/>
+      <c r="AC62" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089951000166468</t>
         </is>
       </c>
@@ -6456,6 +6856,12 @@
       </c>
       <c r="AA63" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB63" s="5" t="inlineStr"/>
+      <c r="AC63" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089961000197247</t>
         </is>
       </c>
@@ -6559,6 +6965,12 @@
       </c>
       <c r="AA64" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB64" s="5" t="inlineStr"/>
+      <c r="AC64" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089971000197252</t>
         </is>
       </c>
@@ -6662,6 +7074,12 @@
       </c>
       <c r="AA65" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB65" s="5" t="inlineStr"/>
+      <c r="AC65" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089981000186398</t>
         </is>
       </c>
@@ -6765,6 +7183,16 @@
       </c>
       <c r="AA66" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB66" s="5" t="inlineStr">
+        <is>
+          <t>[ALTA] Industrialização x retorno: Item 1 (FRASCO IMPRESSO OX 20V 900ML MIX ETERNIZE) é insumo do cliente (CST 41, PIS 49) com CFOP 6124 de industrialização - o mesmo item foi devolvido também na NF 9005 (6902). Retorno de insumo é 5902/6902; como está, R$ 948.00 entra no acumulador de industrialização e na base do PIS/COFINS e do IRPJ/CSLL</t>
+        </is>
+      </c>
+      <c r="AC66" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000089991000116443</t>
         </is>
       </c>
@@ -6868,6 +7296,16 @@
       </c>
       <c r="AA67" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB67" s="5" t="inlineStr">
+        <is>
+          <t>[ALTA] Industrialização x retorno: Item 1 (FRASCO IMPRESSO OX 20V 900ML MIX ETERNIZE) é insumo do cliente (CST 41, PIS 49) com CFOP 5124 de industrialização - o mesmo item foi devolvido também na NF 9002 (5902). Retorno de insumo é 5902/6902; como está, R$ 556.50 entra no acumulador de industrialização e na base do PIS/COFINS e do IRPJ/CSLL</t>
+        </is>
+      </c>
+      <c r="AC67" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090001000116462</t>
         </is>
       </c>
@@ -6971,6 +7409,12 @@
       </c>
       <c r="AA68" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB68" s="5" t="inlineStr"/>
+      <c r="AC68" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090011000116478</t>
         </is>
       </c>
@@ -7074,6 +7518,12 @@
       </c>
       <c r="AA69" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB69" s="5" t="inlineStr"/>
+      <c r="AC69" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090021000116483</t>
         </is>
       </c>
@@ -7177,6 +7627,16 @@
       </c>
       <c r="AA70" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB70" s="5" t="inlineStr">
+        <is>
+          <t>[MÉDIA] CFOP revenda x produção: 4 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+        </is>
+      </c>
+      <c r="AC70" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090031000162296</t>
         </is>
       </c>
@@ -7280,6 +7740,12 @@
       </c>
       <c r="AA71" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB71" s="5" t="inlineStr"/>
+      <c r="AC71" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090041000116496</t>
         </is>
       </c>
@@ -7383,6 +7849,12 @@
       </c>
       <c r="AA72" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB72" s="5" t="inlineStr"/>
+      <c r="AC72" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090051000116507</t>
         </is>
       </c>
@@ -7486,6 +7958,16 @@
       </c>
       <c r="AA73" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB73" s="5" t="inlineStr">
+        <is>
+          <t>[MÉDIA] CFOP revenda x produção: 1 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+        </is>
+      </c>
+      <c r="AC73" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090061000162328</t>
         </is>
       </c>
@@ -7589,6 +8071,12 @@
       </c>
       <c r="AA74" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB74" s="5" t="inlineStr"/>
+      <c r="AC74" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090071000170263</t>
         </is>
       </c>
@@ -7692,6 +8180,12 @@
       </c>
       <c r="AA75" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB75" s="5" t="inlineStr"/>
+      <c r="AC75" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090081000170279</t>
         </is>
       </c>
@@ -7795,6 +8289,16 @@
       </c>
       <c r="AA76" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB76" s="5" t="inlineStr">
+        <is>
+          <t>[MÉDIA] CFOP revenda x produção: 5 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+        </is>
+      </c>
+      <c r="AC76" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090091000162354</t>
         </is>
       </c>
@@ -7898,6 +8402,12 @@
       </c>
       <c r="AA77" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB77" s="5" t="inlineStr"/>
+      <c r="AC77" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090101000217818</t>
         </is>
       </c>
@@ -8001,6 +8511,12 @@
       </c>
       <c r="AA78" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB78" s="5" t="inlineStr"/>
+      <c r="AC78" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090111000162379</t>
         </is>
       </c>
@@ -8104,6 +8620,12 @@
       </c>
       <c r="AA79" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB79" s="5" t="inlineStr"/>
+      <c r="AC79" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090121000217839</t>
         </is>
       </c>
@@ -8207,6 +8729,16 @@
       </c>
       <c r="AA80" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB80" s="5" t="inlineStr">
+        <is>
+          <t>[MÉDIA] CFOP revenda x produção: 2 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+        </is>
+      </c>
+      <c r="AC80" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090131000162390</t>
         </is>
       </c>
@@ -8310,6 +8842,16 @@
       </c>
       <c r="AA81" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB81" s="5" t="inlineStr">
+        <is>
+          <t>[MÉDIA] CFOP revenda x produção: 1 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+        </is>
+      </c>
+      <c r="AC81" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090141000162400</t>
         </is>
       </c>
@@ -8413,6 +8955,12 @@
       </c>
       <c r="AA82" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB82" s="5" t="inlineStr"/>
+      <c r="AC82" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090151000189365</t>
         </is>
       </c>
@@ -8516,6 +9064,12 @@
       </c>
       <c r="AA83" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB83" s="5" t="inlineStr"/>
+      <c r="AC83" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090161000163304</t>
         </is>
       </c>
@@ -8619,6 +9173,16 @@
       </c>
       <c r="AA84" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB84" s="5" t="inlineStr">
+        <is>
+          <t>[BAIXA] Industrialização x retorno: Informações complementares citam a industrialização na NF 9015, que é de FABIANO RODRIGUES AMARAL (CFOP 6101); a do cliente é a NF 9016 - informativo, escriturado como está no XML</t>
+        </is>
+      </c>
+      <c r="AC84" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090171000163310</t>
         </is>
       </c>
@@ -8722,6 +9286,16 @@
       </c>
       <c r="AA85" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB85" s="5" t="inlineStr">
+        <is>
+          <t>[MÉDIA] CFOP revenda x produção: 1 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+        </is>
+      </c>
+      <c r="AC85" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090181000162442</t>
         </is>
       </c>
@@ -8825,6 +9399,16 @@
       </c>
       <c r="AA86" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB86" s="5" t="inlineStr">
+        <is>
+          <t>[MÉDIA] CFOP revenda x produção: 41 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+        </is>
+      </c>
+      <c r="AC86" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090191000162458</t>
         </is>
       </c>
@@ -8928,6 +9512,16 @@
       </c>
       <c r="AA87" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB87" s="5" t="inlineStr">
+        <is>
+          <t>[ALTA] Industrialização x retorno: Item 1 (FRASCO IMPRESSO OX 30V 900ML MIX ETERNIZE) é insumo do cliente (CST 41, PIS 49) com CFOP 6124 de industrialização - o mesmo item foi devolvido também na NF 9026 (6902). Retorno de insumo é 5902/6902; como está, R$ 600.00 entra no acumulador de industrialização e na base do PIS/COFINS e do IRPJ/CSLL</t>
+        </is>
+      </c>
+      <c r="AC87" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090201000116651</t>
         </is>
       </c>
@@ -9031,6 +9625,16 @@
       </c>
       <c r="AA88" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB88" s="5" t="inlineStr">
+        <is>
+          <t>[ALTA] Industrialização x retorno: Item 1 (FRASCO IMPRESSO OX 30V 900ML MIX ETERNIZE) é insumo do cliente (CST 41, PIS 49) com CFOP 5124 de industrialização - o mesmo item foi devolvido também na NF 9024 (5902). Retorno de insumo é 5902/6902; como está, R$ 300.00 entra no acumulador de industrialização e na base do PIS/COFINS e do IRPJ/CSLL</t>
+        </is>
+      </c>
+      <c r="AC88" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090211000116675</t>
         </is>
       </c>
@@ -9134,6 +9738,12 @@
       </c>
       <c r="AA89" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB89" s="5" t="inlineStr"/>
+      <c r="AC89" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090221000192042</t>
         </is>
       </c>
@@ -9237,6 +9847,12 @@
       </c>
       <c r="AA90" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB90" s="5" t="inlineStr"/>
+      <c r="AC90" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090231000116696</t>
         </is>
       </c>
@@ -9340,6 +9956,12 @@
       </c>
       <c r="AA91" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB91" s="5" t="inlineStr"/>
+      <c r="AC91" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090241000116707</t>
         </is>
       </c>
@@ -9443,6 +10065,12 @@
       </c>
       <c r="AA92" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB92" s="5" t="inlineStr"/>
+      <c r="AC92" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090251000116704</t>
         </is>
       </c>
@@ -9546,6 +10174,12 @@
       </c>
       <c r="AA93" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB93" s="5" t="inlineStr"/>
+      <c r="AC93" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090261000116710</t>
         </is>
       </c>
@@ -9649,6 +10283,12 @@
       </c>
       <c r="AA94" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB94" s="5" t="inlineStr"/>
+      <c r="AC94" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090271000116792</t>
         </is>
       </c>
@@ -9752,6 +10392,12 @@
       </c>
       <c r="AA95" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB95" s="5" t="inlineStr"/>
+      <c r="AC95" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090281000116803</t>
         </is>
       </c>
@@ -9855,6 +10501,12 @@
       </c>
       <c r="AA96" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB96" s="5" t="inlineStr"/>
+      <c r="AC96" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090291000186701</t>
         </is>
       </c>
@@ -9958,6 +10610,12 @@
       </c>
       <c r="AA97" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB97" s="5" t="inlineStr"/>
+      <c r="AC97" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090301000186710</t>
         </is>
       </c>
@@ -10061,6 +10719,12 @@
       </c>
       <c r="AA98" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB98" s="5" t="inlineStr"/>
+      <c r="AC98" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090311000119484</t>
         </is>
       </c>
@@ -10164,6 +10828,12 @@
       </c>
       <c r="AA99" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB99" s="5" t="inlineStr"/>
+      <c r="AC99" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090321000119490</t>
         </is>
       </c>
@@ -10267,6 +10937,12 @@
       </c>
       <c r="AA100" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB100" s="5" t="inlineStr"/>
+      <c r="AC100" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090331000116781</t>
         </is>
       </c>
@@ -10370,6 +11046,12 @@
       </c>
       <c r="AA101" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB101" s="5" t="inlineStr"/>
+      <c r="AC101" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090341000116797</t>
         </is>
       </c>
@@ -10473,6 +11155,12 @@
       </c>
       <c r="AA102" s="5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB102" s="5" t="inlineStr"/>
+      <c r="AC102" s="5" t="inlineStr">
+        <is>
           <t>41260933039048000162550010000090351000187314</t>
         </is>
       </c>
@@ -10575,6 +11263,12 @@
         </is>
       </c>
       <c r="AA103" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AB103" s="5" t="inlineStr"/>
+      <c r="AC103" s="5" t="inlineStr">
         <is>
           <t>41260933039048000162550010000090361000187320</t>
         </is>
@@ -10657,6 +11351,8 @@
       <c r="Y104" s="8" t="n"/>
       <c r="Z104" s="8" t="n"/>
       <c r="AA104" s="8" t="n"/>
+      <c r="AB104" s="8" t="n"/>
+      <c r="AC104" s="8" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
@@ -10703,8 +11399,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:AA103"/>
-  <conditionalFormatting sqref="A5:AA103">
+  <autoFilter ref="A4:AC103"/>
+  <conditionalFormatting sqref="A5:AC103">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E5="Cancelada"</formula>
     </cfRule>

</xml_diff>